<commit_message>
Add import-update feature with medical check logic
</commit_message>
<xml_diff>
--- a/app/MAU RP XUAT BAO CAO/IMPORT MDK UPLOAD THONG TIN HV.xlsx
+++ b/app/MAU RP XUAT BAO CAO/IMPORT MDK UPLOAD THONG TIN HV.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\web-giao-vucd\app\api\import-update\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\web-giao-vucd\app\MAU RP XUAT BAO CAO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBAA9289-FF70-4072-9B17-73EBE0453188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA495D33-8899-4D8D-8DA4-62BB3D5A1192}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
   <si>
     <t>ma_dk</t>
   </si>
@@ -55,6 +55,12 @@
   </si>
   <si>
     <t>0656562454</t>
+  </si>
+  <si>
+    <t>giao_vien</t>
+  </si>
+  <si>
+    <t>ctv</t>
   </si>
 </sst>
 </file>
@@ -396,16 +402,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="38.125" customWidth="1"/>
     <col min="2" max="2" width="25.75" style="6" customWidth="1"/>
     <col min="3" max="3" width="18.75" customWidth="1"/>
-    <col min="4" max="4" width="30.375" customWidth="1"/>
+    <col min="4" max="5" width="21.125" customWidth="1"/>
+    <col min="6" max="6" width="30.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="30" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -416,10 +423,16 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -429,11 +442,13 @@
       <c r="C2" s="3">
         <v>46114</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
@@ -443,7 +458,9 @@
       <c r="C3" s="3">
         <v>46122</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="2" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>